<commit_message>
#3 (Added Sheet 1000pcs Cost for Main Board)
</commit_message>
<xml_diff>
--- a/Design Files/LLR-05U (Advance Version)/Main Board/BOM/eSpark BOM LLR-05U (Main-Board).xlsx
+++ b/Design Files/LLR-05U (Advance Version)/Main Board/BOM/eSpark BOM LLR-05U (Main-Board).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20410"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Main Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8165E5-A034-4592-A546-8D1C8711EEB1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F3A287-37B8-496D-8D36-1DBDD696B30A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -876,6 +876,12 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -898,12 +904,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1335,15 +1335,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="44"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="46"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1368,7 +1368,7 @@
       <c r="P2" s="33"/>
       <c r="Q2" s="33"/>
       <c r="R2" s="33"/>
-      <c r="S2" s="47"/>
+      <c r="S2" s="49"/>
     </row>
     <row r="3" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -1393,7 +1393,7 @@
       <c r="P3" s="25"/>
       <c r="Q3" s="25"/>
       <c r="R3" s="25"/>
-      <c r="S3" s="48"/>
+      <c r="S3" s="50"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1414,7 +1414,7 @@
       <c r="P4" s="25"/>
       <c r="Q4" s="25"/>
       <c r="R4" s="25"/>
-      <c r="S4" s="48"/>
+      <c r="S4" s="50"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1435,7 +1435,7 @@
       <c r="P5" s="36"/>
       <c r="Q5" s="36"/>
       <c r="R5" s="36"/>
-      <c r="S5" s="48"/>
+      <c r="S5" s="50"/>
     </row>
     <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -1456,7 +1456,7 @@
       <c r="P6" s="36"/>
       <c r="Q6" s="36"/>
       <c r="R6" s="36"/>
-      <c r="S6" s="49"/>
+      <c r="S6" s="51"/>
     </row>
     <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -1554,7 +1554,7 @@
       <c r="N8" s="14">
         <v>10</v>
       </c>
-      <c r="O8" s="50" t="s">
+      <c r="O8" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P8" s="15">
@@ -1608,7 +1608,7 @@
       <c r="N9" s="21">
         <v>20</v>
       </c>
-      <c r="O9" s="51" t="s">
+      <c r="O9" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P9" s="22">
@@ -1662,7 +1662,7 @@
       <c r="N10" s="14">
         <v>20</v>
       </c>
-      <c r="O10" s="50" t="s">
+      <c r="O10" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P10" s="15">
@@ -1716,7 +1716,7 @@
       <c r="N11" s="21">
         <v>100</v>
       </c>
-      <c r="O11" s="51" t="s">
+      <c r="O11" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P11" s="22">
@@ -1770,7 +1770,7 @@
       <c r="N12" s="14">
         <v>100</v>
       </c>
-      <c r="O12" s="50" t="s">
+      <c r="O12" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P12" s="15">
@@ -1824,7 +1824,7 @@
       <c r="N13" s="21">
         <v>10</v>
       </c>
-      <c r="O13" s="51" t="s">
+      <c r="O13" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P13" s="22">
@@ -1878,7 +1878,7 @@
       <c r="N14" s="14">
         <v>5</v>
       </c>
-      <c r="O14" s="50" t="s">
+      <c r="O14" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P14" s="15">
@@ -1932,7 +1932,7 @@
       <c r="N15" s="21">
         <v>5</v>
       </c>
-      <c r="O15" s="51" t="s">
+      <c r="O15" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P15" s="22">
@@ -1986,7 +1986,7 @@
       <c r="N16" s="14">
         <v>50</v>
       </c>
-      <c r="O16" s="50" t="s">
+      <c r="O16" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P16" s="15">
@@ -2040,7 +2040,7 @@
       <c r="N17" s="21">
         <v>100</v>
       </c>
-      <c r="O17" s="51" t="s">
+      <c r="O17" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P17" s="22">
@@ -2094,7 +2094,7 @@
       <c r="N18" s="14">
         <v>100</v>
       </c>
-      <c r="O18" s="50" t="s">
+      <c r="O18" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P18" s="15">
@@ -2148,7 +2148,7 @@
       <c r="N19" s="21">
         <v>20</v>
       </c>
-      <c r="O19" s="51" t="s">
+      <c r="O19" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P19" s="22">
@@ -2202,7 +2202,7 @@
       <c r="N20" s="14">
         <v>20</v>
       </c>
-      <c r="O20" s="50" t="s">
+      <c r="O20" s="43" t="s">
         <v>118</v>
       </c>
       <c r="P20" s="15">
@@ -2250,7 +2250,7 @@
       <c r="N21" s="21">
         <v>5</v>
       </c>
-      <c r="O21" s="51" t="s">
+      <c r="O21" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P21" s="22">
@@ -2292,7 +2292,7 @@
       <c r="N22" s="14">
         <v>5</v>
       </c>
-      <c r="O22" s="50" t="s">
+      <c r="O22" s="43" t="s">
         <v>121</v>
       </c>
       <c r="P22" s="15">
@@ -2346,7 +2346,7 @@
       <c r="N23" s="21">
         <v>10</v>
       </c>
-      <c r="O23" s="51" t="s">
+      <c r="O23" s="44" t="s">
         <v>118</v>
       </c>
       <c r="P23" s="22">
@@ -2373,11 +2373,11 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
-      <c r="N24" s="45" t="s">
+      <c r="N24" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="O24" s="46"/>
-      <c r="P24" s="46"/>
+      <c r="O24" s="48"/>
+      <c r="P24" s="48"/>
       <c r="Q24" s="18">
         <f>SUM(Q8:Q23)</f>
         <v>24.337999999999997</v>
@@ -2399,11 +2399,11 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
-      <c r="N25" s="45" t="s">
+      <c r="N25" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="O25" s="46"/>
-      <c r="P25" s="46"/>
+      <c r="O25" s="48"/>
+      <c r="P25" s="48"/>
       <c r="Q25" s="19">
         <f>Q24/5</f>
         <v>4.8675999999999995</v>
@@ -2481,15 +2481,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="44"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="46"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2514,7 +2514,7 @@
       <c r="P2" s="33"/>
       <c r="Q2" s="33"/>
       <c r="R2" s="33"/>
-      <c r="S2" s="47"/>
+      <c r="S2" s="49"/>
     </row>
     <row r="3" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -2539,7 +2539,7 @@
       <c r="P3" s="25"/>
       <c r="Q3" s="25"/>
       <c r="R3" s="25"/>
-      <c r="S3" s="48"/>
+      <c r="S3" s="50"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2560,7 +2560,7 @@
       <c r="P4" s="25"/>
       <c r="Q4" s="25"/>
       <c r="R4" s="25"/>
-      <c r="S4" s="48"/>
+      <c r="S4" s="50"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2581,7 +2581,7 @@
       <c r="P5" s="36"/>
       <c r="Q5" s="36"/>
       <c r="R5" s="36"/>
-      <c r="S5" s="48"/>
+      <c r="S5" s="50"/>
     </row>
     <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -2602,7 +2602,7 @@
       <c r="P6" s="36"/>
       <c r="Q6" s="36"/>
       <c r="R6" s="36"/>
-      <c r="S6" s="49"/>
+      <c r="S6" s="51"/>
     </row>
     <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -2697,14 +2697,18 @@
         <f>L8*1000</f>
         <v>1000</v>
       </c>
-      <c r="N8" s="14"/>
-      <c r="O8" s="50" t="s">
+      <c r="N8" s="14">
+        <v>1000</v>
+      </c>
+      <c r="O8" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P8" s="15"/>
+      <c r="P8" s="15">
+        <v>3.8699999999999998E-2</v>
+      </c>
       <c r="Q8" s="15">
         <f>P8*N8</f>
-        <v>0</v>
+        <v>38.699999999999996</v>
       </c>
       <c r="R8" s="14"/>
       <c r="S8" s="20"/>
@@ -2747,14 +2751,18 @@
         <f t="shared" ref="M9:M23" si="1">L9*1000</f>
         <v>1000</v>
       </c>
-      <c r="N9" s="21"/>
-      <c r="O9" s="51" t="s">
+      <c r="N9" s="21">
+        <v>1000</v>
+      </c>
+      <c r="O9" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P9" s="22"/>
+      <c r="P9" s="22">
+        <v>1.14E-2</v>
+      </c>
       <c r="Q9" s="22">
         <f t="shared" ref="Q9" si="2">P9*N9</f>
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="R9" s="21"/>
       <c r="S9" s="21"/>
@@ -2797,14 +2805,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N10" s="14"/>
-      <c r="O10" s="50" t="s">
+      <c r="N10" s="14">
+        <v>2000</v>
+      </c>
+      <c r="O10" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P10" s="15"/>
+      <c r="P10" s="15">
+        <v>1.4200000000000001E-2</v>
+      </c>
       <c r="Q10" s="15">
         <f>P10*N10</f>
-        <v>0</v>
+        <v>28.400000000000002</v>
       </c>
       <c r="R10" s="14"/>
       <c r="S10" s="20"/>
@@ -2847,14 +2859,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N11" s="21"/>
-      <c r="O11" s="51" t="s">
+      <c r="N11" s="21">
+        <v>1000</v>
+      </c>
+      <c r="O11" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P11" s="22"/>
+      <c r="P11" s="22">
+        <v>5.5999999999999999E-3</v>
+      </c>
       <c r="Q11" s="22">
         <f t="shared" ref="Q11" si="3">P11*N11</f>
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="R11" s="21"/>
       <c r="S11" s="21"/>
@@ -2897,14 +2913,18 @@
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
-      <c r="N12" s="14"/>
-      <c r="O12" s="50" t="s">
+      <c r="N12" s="14">
+        <v>3000</v>
+      </c>
+      <c r="O12" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P12" s="15"/>
+      <c r="P12" s="15">
+        <v>4.3E-3</v>
+      </c>
       <c r="Q12" s="15">
         <f>P12*N12</f>
-        <v>0</v>
+        <v>12.9</v>
       </c>
       <c r="R12" s="14"/>
       <c r="S12" s="20"/>
@@ -2947,14 +2967,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N13" s="21"/>
-      <c r="O13" s="51" t="s">
+      <c r="N13" s="21">
+        <v>2000</v>
+      </c>
+      <c r="O13" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P13" s="22"/>
+      <c r="P13" s="22">
+        <v>0.16339999999999999</v>
+      </c>
       <c r="Q13" s="22">
         <f t="shared" ref="Q13" si="4">P13*N13</f>
-        <v>0</v>
+        <v>326.79999999999995</v>
       </c>
       <c r="R13" s="21"/>
       <c r="S13" s="21"/>
@@ -2997,14 +3021,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N14" s="14"/>
-      <c r="O14" s="50" t="s">
+      <c r="N14" s="14">
+        <v>1000</v>
+      </c>
+      <c r="O14" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P14" s="15"/>
+      <c r="P14" s="15">
+        <v>0.11119999999999999</v>
+      </c>
       <c r="Q14" s="15">
         <f>P14*N14</f>
-        <v>0</v>
+        <v>111.19999999999999</v>
       </c>
       <c r="R14" s="14"/>
       <c r="S14" s="20"/>
@@ -3047,14 +3075,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N15" s="21"/>
-      <c r="O15" s="51" t="s">
+      <c r="N15" s="21">
+        <v>1000</v>
+      </c>
+      <c r="O15" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P15" s="22"/>
+      <c r="P15" s="22">
+        <v>4.3499999999999997E-2</v>
+      </c>
       <c r="Q15" s="22">
         <f t="shared" ref="Q15" si="5">P15*N15</f>
-        <v>0</v>
+        <v>43.5</v>
       </c>
       <c r="R15" s="21"/>
       <c r="S15" s="21"/>
@@ -3097,14 +3129,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N16" s="14"/>
-      <c r="O16" s="50" t="s">
+      <c r="N16" s="14">
+        <v>2000</v>
+      </c>
+      <c r="O16" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P16" s="15"/>
+      <c r="P16" s="15">
+        <v>6.7999999999999996E-3</v>
+      </c>
       <c r="Q16" s="15">
         <f>P16*N16</f>
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="R16" s="14"/>
       <c r="S16" s="20"/>
@@ -3147,14 +3183,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N17" s="21"/>
-      <c r="O17" s="51" t="s">
+      <c r="N17" s="21">
+        <v>1000</v>
+      </c>
+      <c r="O17" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P17" s="22"/>
+      <c r="P17" s="22">
+        <v>1.2999999999999999E-3</v>
+      </c>
       <c r="Q17" s="22">
         <f t="shared" ref="Q17" si="6">P17*N17</f>
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="R17" s="21"/>
       <c r="S17" s="21"/>
@@ -3197,14 +3237,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N18" s="14"/>
-      <c r="O18" s="50" t="s">
+      <c r="N18" s="14">
+        <v>2000</v>
+      </c>
+      <c r="O18" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P18" s="15"/>
+      <c r="P18" s="15">
+        <v>2.2000000000000001E-3</v>
+      </c>
       <c r="Q18" s="15">
         <f>P18*N18</f>
-        <v>0</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="R18" s="14"/>
       <c r="S18" s="20"/>
@@ -3247,14 +3291,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N19" s="21"/>
-      <c r="O19" s="51" t="s">
+      <c r="N19" s="21">
+        <v>2000</v>
+      </c>
+      <c r="O19" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P19" s="22"/>
+      <c r="P19" s="22">
+        <v>1.34E-2</v>
+      </c>
       <c r="Q19" s="22">
         <f t="shared" ref="Q19" si="7">P19*N19</f>
-        <v>0</v>
+        <v>26.8</v>
       </c>
       <c r="R19" s="21"/>
       <c r="S19" s="21"/>
@@ -3297,14 +3345,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N20" s="14"/>
-      <c r="O20" s="50" t="s">
+      <c r="N20" s="14">
+        <v>2000</v>
+      </c>
+      <c r="O20" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="P20" s="15"/>
+      <c r="P20" s="15">
+        <v>1.61E-2</v>
+      </c>
       <c r="Q20" s="15">
         <f>P20*N20</f>
-        <v>0</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="R20" s="14"/>
       <c r="S20" s="20"/>
@@ -3341,14 +3393,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N21" s="21"/>
-      <c r="O21" s="51" t="s">
+      <c r="N21" s="21">
+        <v>1000</v>
+      </c>
+      <c r="O21" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P21" s="22"/>
+      <c r="P21" s="22">
+        <v>0.4224</v>
+      </c>
       <c r="Q21" s="22">
         <f t="shared" ref="Q21" si="8">P21*N21</f>
-        <v>0</v>
+        <v>422.4</v>
       </c>
       <c r="R21" s="21"/>
       <c r="S21" s="21"/>
@@ -3379,14 +3435,18 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N22" s="14"/>
-      <c r="O22" s="50" t="s">
+      <c r="N22" s="14">
+        <v>1000</v>
+      </c>
+      <c r="O22" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="P22" s="15"/>
+      <c r="P22" s="15">
+        <v>1.46</v>
+      </c>
       <c r="Q22" s="15">
         <f>P22*N22</f>
-        <v>0</v>
+        <v>1460</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="20"/>
@@ -3429,14 +3489,18 @@
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="N23" s="21"/>
-      <c r="O23" s="51" t="s">
+      <c r="N23" s="21">
+        <v>2000</v>
+      </c>
+      <c r="O23" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="P23" s="22"/>
+      <c r="P23" s="22">
+        <v>7.5200000000000003E-2</v>
+      </c>
       <c r="Q23" s="22">
         <f t="shared" ref="Q23" si="9">P23*N23</f>
-        <v>0</v>
+        <v>150.4</v>
       </c>
       <c r="R23" s="21"/>
       <c r="S23" s="21"/>
@@ -3455,14 +3519,14 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
-      <c r="N24" s="45" t="s">
+      <c r="N24" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="O24" s="46"/>
-      <c r="P24" s="46"/>
+      <c r="O24" s="48"/>
+      <c r="P24" s="48"/>
       <c r="Q24" s="18">
         <f>SUM(Q8:Q23)</f>
-        <v>0</v>
+        <v>2689.6</v>
       </c>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
@@ -3481,14 +3545,14 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
-      <c r="N25" s="45" t="s">
+      <c r="N25" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="O25" s="46"/>
-      <c r="P25" s="46"/>
+      <c r="O25" s="48"/>
+      <c r="P25" s="48"/>
       <c r="Q25" s="19">
         <f>Q24/1000</f>
-        <v>0</v>
+        <v>2.6896</v>
       </c>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -3522,6 +3586,7 @@
     <hyperlink ref="O23" r:id="rId16" xr:uid="{E1565B14-DA57-48A0-8D54-B71EA998B58D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>